<commit_message>
Write the DSR in the first person singular
It is submitted under one name, so "we" was the wrong voice. Where the plural
was doing real work it is now named instead of implied: "our farmers" means
Indian farmers, "our users" means SmartKisan users, and "a product we sell"
means one the company sells. Those are not the writer and should not have been
carried by the same pronoun as the ones that were.

The reasons section reads better for it. "Running two at once was tried" hid
who tried it and what it cost them; "I tried running two at once" is the
sentence a reader wants when the question on the table is where three days
went.

Adds a "Prepared by" line under the sub-title, which moves the column headings
to row 5 -- now a constant rather than three separate hardcoded 4s and an "A5".
</commit_message>
<xml_diff>
--- a/SmartKisan_DSR_2026-09-10_to_09-14.xlsx
+++ b/SmartKisan_DSR_2026-09-10_to_09-14.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="9">
+  <fonts count="10">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -32,6 +32,10 @@
     </font>
     <font>
       <i val="1"/>
+      <color rgb="00555555"/>
+      <sz val="10"/>
+    </font>
+    <font>
       <color rgb="00555555"/>
       <sz val="10"/>
     </font>
@@ -110,7 +114,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -118,33 +122,36 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -512,7 +519,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G54"/>
+  <dimension ref="A1:G55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -538,749 +545,731 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="28" customHeight="1">
-      <c r="A4" s="3" t="inlineStr">
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Prepared by: Karishma</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="28" customHeight="1">
+      <c r="A5" s="4" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B5" s="4" t="inlineStr">
         <is>
           <t>Task Category</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C5" s="4" t="inlineStr">
         <is>
           <t>Detailed Task Description</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D5" s="4" t="inlineStr">
         <is>
           <t>Deliverables / Artifacts</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="E5" s="4" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="F5" s="4" t="inlineStr">
         <is>
           <t>Hours Spent</t>
         </is>
       </c>
-      <c r="G4" s="3" t="inlineStr">
+      <c r="G5" s="4" t="inlineStr">
         <is>
           <t>Remarks &amp; Notes</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="4" t="inlineStr">
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
         <is>
           <t>2026-09-10</t>
         </is>
       </c>
-      <c r="B5" s="4" t="inlineStr">
+      <c r="B6" s="5" t="inlineStr">
         <is>
           <t>Disease Detection - Measurement</t>
         </is>
       </c>
-      <c r="C5" s="4" t="inlineStr">
+      <c r="C6" s="5" t="inlineStr">
         <is>
           <t>Measured the model running in the app against 1,581 photographs it had never seen, taken in real fields rather than in a laboratory. The figure quoted until now came from images of the same kind it learned from, which reports memorisation rather than usefulness.</t>
         </is>
       </c>
-      <c r="D5" s="4" t="inlineStr">
+      <c r="D6" s="5" t="inlineStr">
         <is>
           <t>evaluate_india_model.py</t>
         </is>
       </c>
-      <c r="E5" s="5" t="inlineStr">
+      <c r="E6" s="6" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="F5" s="6" t="n">
+      <c r="F6" s="7" t="n">
         <v>1.5</v>
       </c>
-      <c r="G5" s="4" t="inlineStr">
+      <c r="G6" s="5" t="inlineStr">
         <is>
           <t>Named the disease correctly in 28 photographs out of 100, and the crop in 49. Worse, 42 healthy plants out of every 100 were reported as diseased - a farmer sent to buy a spray he does not need.</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="4" t="inlineStr">
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
         <is>
           <t>2026-09-10</t>
         </is>
       </c>
-      <c r="B6" s="4" t="inlineStr">
+      <c r="B7" s="5" t="inlineStr">
         <is>
           <t>Disease Detection - Root Cause</t>
         </is>
       </c>
-      <c r="C6" s="4" t="inlineStr">
-        <is>
-          <t>Examined what the model had actually been taught. 16 of its 38 disease classes are apple, grape, cherry, peach, blueberry, raspberry and strawberry: temperate orchard and berry crops our farmers do not grow. It had no wheat and no rice at all.</t>
-        </is>
-      </c>
-      <c r="D6" s="4" t="inlineStr">
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>Examined what the model had actually been taught. 16 of its 38 disease classes are apple, grape, cherry, peach, blueberry, raspberry and strawberry: temperate orchard and berry crops Indian farmers do not grow. It had no wheat and no rice at all.</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
         <is>
           <t>classes_india.py</t>
         </is>
       </c>
-      <c r="E6" s="5" t="inlineStr">
+      <c r="E7" s="6" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="F6" s="6" t="n">
+      <c r="F7" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="G6" s="4" t="inlineStr">
+      <c r="G7" s="5" t="inlineStr">
         <is>
           <t>A farmer photographing wheat was receiving a confident answer about a tomato, because wheat was not an answer the model could give. No amount of tuning fixes a wrong list of crops.</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="4" t="inlineStr">
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
         <is>
           <t>2026-09-10</t>
         </is>
       </c>
-      <c r="B7" s="4" t="inlineStr">
+      <c r="B8" s="5" t="inlineStr">
         <is>
           <t>Training Data - Sourcing and Licensing</t>
         </is>
       </c>
-      <c r="C7" s="4" t="inlineStr">
+      <c r="C8" s="5" t="inlineStr">
         <is>
           <t>Selected replacement training collections covering rice, wheat and field-grown potato, maize and tomato, and checked the licence on each one before downloading it.</t>
         </is>
       </c>
-      <c r="D7" s="4" t="inlineStr">
+      <c r="D8" s="5" t="inlineStr">
         <is>
           <t>Four public collections, licences recorded</t>
         </is>
       </c>
-      <c r="E7" s="5" t="inlineStr">
+      <c r="E8" s="6" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="F7" s="6" t="n">
+      <c r="F8" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="G7" s="4" t="inlineStr">
-        <is>
-          <t>One good multi-crop set from Bangladesh was rejected: its licence forbids commercial use, so it cannot sit inside a product we sell. Cheaper to find that now than after it is in a shipped model.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="4" t="inlineStr">
+      <c r="G8" s="5" t="inlineStr">
+        <is>
+          <t>One good multi-crop set from Bangladesh was rejected: its licence forbids commercial use, so it cannot sit inside a product the company sells. Cheaper to find that now than after it is in a shipped model.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
         <is>
           <t>2026-09-10</t>
         </is>
       </c>
-      <c r="B8" s="4" t="inlineStr">
+      <c r="B9" s="5" t="inlineStr">
         <is>
           <t>Training Data - Download</t>
         </is>
       </c>
-      <c r="C8" s="4" t="inlineStr">
+      <c r="C9" s="5" t="inlineStr">
         <is>
           <t>Downloaded roughly 1.5 GB of imagery across the four collections.</t>
         </is>
       </c>
-      <c r="D8" s="4" t="inlineStr">
+      <c r="D9" s="5" t="inlineStr">
         <is>
           <t>dataset/ (not committed)</t>
         </is>
       </c>
-      <c r="E8" s="5" t="inlineStr">
+      <c r="E9" s="6" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="F8" s="6" t="n">
+      <c r="F9" s="7" t="n">
         <v>1.5</v>
       </c>
-      <c r="G8" s="4" t="inlineStr">
+      <c r="G9" s="5" t="inlineStr">
         <is>
           <t>One host began refusing requests for downloading too quickly and the download had to be slowed and restarted from the beginning. Unavoidable, and it cost about half of this time.</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="7" t="inlineStr"/>
-      <c r="B9" s="8" t="inlineStr">
+    <row r="10">
+      <c r="A10" s="8" t="inlineStr"/>
+      <c r="B10" s="9" t="inlineStr">
         <is>
           <t>Thursday 10 September - total</t>
         </is>
       </c>
-      <c r="C9" s="7" t="inlineStr"/>
-      <c r="D9" s="7" t="inlineStr"/>
-      <c r="E9" s="7" t="inlineStr"/>
-      <c r="F9" s="9" t="n">
+      <c r="C10" s="8" t="inlineStr"/>
+      <c r="D10" s="8" t="inlineStr"/>
+      <c r="E10" s="8" t="inlineStr"/>
+      <c r="F10" s="10" t="n">
         <v>6</v>
       </c>
-      <c r="G9" s="7" t="inlineStr"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="4" t="inlineStr">
+      <c r="G10" s="8" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
         <is>
           <t>2026-09-11</t>
         </is>
       </c>
-      <c r="B10" s="4" t="inlineStr">
+      <c r="B11" s="5" t="inlineStr">
         <is>
           <t>Disease Detection - New Crop List</t>
         </is>
       </c>
-      <c r="C10" s="4" t="inlineStr">
+      <c r="C11" s="5" t="inlineStr">
         <is>
           <t>Rebuilt the list of crops and diseases the model can name: 32 classes across 9 crops. Removed the 16 orchard and berry classes, added rice, wheat and field-grown potato, maize and tomato.</t>
         </is>
       </c>
-      <c r="D10" s="4" t="inlineStr">
+      <c r="D11" s="5" t="inlineStr">
         <is>
           <t>classes_india.py, finetune_india.py</t>
         </is>
       </c>
-      <c r="E10" s="5" t="inlineStr">
+      <c r="E11" s="6" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="F10" s="6" t="n">
+      <c r="F11" s="7" t="n">
         <v>1.5</v>
       </c>
-      <c r="G10" s="4" t="inlineStr">
+      <c r="G11" s="5" t="inlineStr">
         <is>
           <t>Caught a trap while doing this. Maize and tomato both have folders named healthy and leaf blight in one dataset. Loaded carelessly, maize disease would have been taught as tomato disease with no error reported anywhere - it would only have shown up later as a model that is wrong for no visible reason.</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="4" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
         <is>
           <t>2026-09-11</t>
         </is>
       </c>
-      <c r="B11" s="4" t="inlineStr">
+      <c r="B12" s="5" t="inlineStr">
         <is>
           <t>Disease Detection - Design Comparison</t>
         </is>
       </c>
-      <c r="C11" s="4" t="inlineStr">
+      <c r="C12" s="5" t="inlineStr">
         <is>
           <t>Compared two model designs on identical data before committing to one, rather than assuming the newer one is better.</t>
         </is>
       </c>
-      <c r="D11" s="4" t="inlineStr">
+      <c r="D12" s="5" t="inlineStr">
         <is>
           <t>finetune_india.py (--arch)</t>
         </is>
       </c>
-      <c r="E11" s="5" t="inlineStr">
+      <c r="E12" s="6" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="F11" s="6" t="n">
+      <c r="F12" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="G11" s="4" t="inlineStr">
+      <c r="G12" s="5" t="inlineStr">
         <is>
           <t>58.1% against 61.9% on field photographs. Kept the better one. Worth the hour: the choice is made once and everything afterwards is built on top of it.</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="4" t="inlineStr">
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
         <is>
           <t>2026-09-11</t>
         </is>
       </c>
-      <c r="B12" s="4" t="inlineStr">
+      <c r="B13" s="5" t="inlineStr">
         <is>
           <t>Disease Detection - First Full Training Run</t>
         </is>
       </c>
-      <c r="C12" s="4" t="inlineStr">
+      <c r="C13" s="5" t="inlineStr">
         <is>
           <t>Trained the model on the new crop list: 20,777 training images, 78% of them photographed in real fields rather than in a laboratory.</t>
         </is>
       </c>
-      <c r="D12" s="4" t="inlineStr">
+      <c r="D13" s="5" t="inlineStr">
         <is>
           <t>india_model.tflite, class_labels_india.json</t>
         </is>
       </c>
-      <c r="E12" s="5" t="inlineStr">
+      <c r="E13" s="6" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="F12" s="6" t="n">
+      <c r="F13" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="G12" s="4" t="inlineStr">
-        <is>
-          <t>85.9% overall, and rice and wheat work for the first time. But three crops were still weak - tomato 44%, potato 50%, maize 65%. Those are the crops our users grow most, so this was not shippable.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="4" t="inlineStr">
+      <c r="G13" s="5" t="inlineStr">
+        <is>
+          <t>85.9% overall, and rice and wheat work for the first time. But three crops were still weak - tomato 44%, potato 50%, maize 65%. Those are the crops most SmartKisan users grow, so this was not shippable.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
         <is>
           <t>2026-09-11</t>
         </is>
       </c>
-      <c r="B13" s="4" t="inlineStr">
+      <c r="B14" s="5" t="inlineStr">
         <is>
           <t>Disease Detection - Service Prepared</t>
         </is>
       </c>
-      <c r="C13" s="4" t="inlineStr">
+      <c r="C14" s="5" t="inlineStr">
         <is>
           <t>Rewrote the service that answers the app so it carries treatment advice for rice and wheat, and reads the image size from the model rather than assuming the old one.</t>
         </is>
       </c>
-      <c r="D13" s="4" t="inlineStr">
+      <c r="D14" s="5" t="inlineStr">
         <is>
           <t>huggingface_india/app.py</t>
         </is>
       </c>
-      <c r="E13" s="5" t="inlineStr">
+      <c r="E14" s="6" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="F13" s="6" t="n">
+      <c r="F14" s="7" t="n">
         <v>0.5</v>
       </c>
-      <c r="G13" s="4" t="inlineStr">
+      <c r="G14" s="5" t="inlineStr">
         <is>
           <t>Rice bacterial blight and rice tungro deliberately advise no spray - neither responds to one, and recommending a chemical that cannot work costs the farmer money for nothing.</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="7" t="inlineStr"/>
-      <c r="B14" s="8" t="inlineStr">
+    <row r="15">
+      <c r="A15" s="8" t="inlineStr"/>
+      <c r="B15" s="9" t="inlineStr">
         <is>
           <t>Friday 11 September - total</t>
         </is>
       </c>
-      <c r="C14" s="7" t="inlineStr"/>
-      <c r="D14" s="7" t="inlineStr"/>
-      <c r="E14" s="7" t="inlineStr"/>
-      <c r="F14" s="9" t="n">
+      <c r="C15" s="8" t="inlineStr"/>
+      <c r="D15" s="8" t="inlineStr"/>
+      <c r="E15" s="8" t="inlineStr"/>
+      <c r="F15" s="10" t="n">
         <v>6</v>
       </c>
-      <c r="G14" s="7" t="inlineStr"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="4" t="inlineStr">
+      <c r="G15" s="8" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
         <is>
           <t>2026-09-12</t>
         </is>
       </c>
-      <c r="B15" s="4" t="inlineStr">
+      <c r="B16" s="5" t="inlineStr">
         <is>
           <t>Disease Detection - First Attempt at the Weak Crops</t>
         </is>
       </c>
-      <c r="C15" s="4" t="inlineStr">
+      <c r="C16" s="5" t="inlineStr">
         <is>
           <t>Tried to lift tomato, potato and maize by giving the model more laboratory photographs of those three crops.</t>
         </is>
       </c>
-      <c r="D15" s="4" t="inlineStr">
+      <c r="D16" s="5" t="inlineStr">
         <is>
           <t>finetune_india.py (rebalanced run)</t>
         </is>
       </c>
-      <c r="E15" s="10" t="inlineStr">
+      <c r="E16" s="11" t="inlineStr">
         <is>
           <t>Investigated - Not Adopted</t>
         </is>
       </c>
-      <c r="F15" s="6" t="n">
+      <c r="F16" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="G15" s="4" t="inlineStr">
+      <c r="G16" s="5" t="inlineStr">
         <is>
           <t>It made tomato worse: 44% down to 38%. Run discarded. Recorded in the code beside the setting it concerns, so it is not tried again.</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="4" t="inlineStr">
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
         <is>
           <t>2026-09-12</t>
         </is>
       </c>
-      <c r="B16" s="4" t="inlineStr">
+      <c r="B17" s="5" t="inlineStr">
         <is>
           <t>Disease Detection - Error Analysis</t>
         </is>
       </c>
-      <c r="C16" s="4" t="inlineStr">
+      <c r="C17" s="5" t="inlineStr">
         <is>
           <t>Instead of guessing at a second attempt, examined exactly which photographs the model was getting wrong and what it answered instead.</t>
         </is>
       </c>
-      <c r="D16" s="4" t="inlineStr">
+      <c r="D17" s="5" t="inlineStr">
         <is>
           <t>evaluate_india_model.py</t>
         </is>
       </c>
-      <c r="E16" s="5" t="inlineStr">
+      <c r="E17" s="6" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="F16" s="6" t="n">
+      <c r="F17" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="G16" s="4" t="inlineStr">
+      <c r="G17" s="5" t="inlineStr">
         <is>
           <t>33 of the 39 tomato mistakes were one tomato disease mistaken for another. The model knew it was a tomato; it could not tell the diseases apart in field conditions. That is why more laboratory photographs failed, and it pointed straight at the real fix.</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="4" t="inlineStr">
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
         <is>
           <t>2026-09-12</t>
         </is>
       </c>
-      <c r="B17" s="4" t="inlineStr">
+      <c r="B18" s="5" t="inlineStr">
         <is>
           <t>Training Data - Corrupt Files</t>
         </is>
       </c>
-      <c r="C17" s="4" t="inlineStr">
+      <c r="C18" s="5" t="inlineStr">
         <is>
           <t>A training run died partway with a corrupt image error that did not name the file. Wrote a tool to find them by opening every image two different ways.</t>
         </is>
       </c>
-      <c r="D17" s="4" t="inlineStr">
+      <c r="D18" s="5" t="inlineStr">
         <is>
           <t>find_bad_images.py</t>
         </is>
       </c>
-      <c r="E17" s="5" t="inlineStr">
+      <c r="E18" s="6" t="inlineStr">
         <is>
           <t>Fixed</t>
         </is>
       </c>
-      <c r="F17" s="6" t="n">
+      <c r="F18" s="7" t="n">
         <v>0.5</v>
       </c>
-      <c r="G17" s="4" t="inlineStr">
+      <c r="G18" s="5" t="inlineStr">
         <is>
           <t>96 broken image files in one download. Skipped by name, so a run does not stop on them and the rest of the collection is still used.</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="4" t="inlineStr">
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
         <is>
           <t>2026-09-12</t>
         </is>
       </c>
-      <c r="B18" s="4" t="inlineStr">
+      <c r="B19" s="5" t="inlineStr">
         <is>
           <t>Disease Detection - Final Training Run</t>
         </is>
       </c>
-      <c r="C18" s="4" t="inlineStr">
+      <c r="C19" s="5" t="inlineStr">
         <is>
           <t>Retrained with real field photographs of the three weak crops instead of more laboratory ones.</t>
         </is>
       </c>
-      <c r="D18" s="4" t="inlineStr">
+      <c r="D19" s="5" t="inlineStr">
         <is>
           <t>india_model.tflite (final)</t>
         </is>
       </c>
-      <c r="E18" s="5" t="inlineStr">
+      <c r="E19" s="6" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="F18" s="6" t="n">
+      <c r="F19" s="7" t="n">
         <v>2.5</v>
       </c>
-      <c r="G18" s="4" t="inlineStr">
+      <c r="G19" s="5" t="inlineStr">
         <is>
           <t>Tomato 44% to 88%, potato 50% to 86%, maize 65% to 82%. Overall 87%. This is the model now in the app.</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="7" t="inlineStr"/>
-      <c r="B19" s="8" t="inlineStr">
+    <row r="20">
+      <c r="A20" s="8" t="inlineStr"/>
+      <c r="B20" s="9" t="inlineStr">
         <is>
           <t>Saturday 12 September - total</t>
         </is>
       </c>
-      <c r="C19" s="7" t="inlineStr"/>
-      <c r="D19" s="7" t="inlineStr"/>
-      <c r="E19" s="7" t="inlineStr"/>
-      <c r="F19" s="9" t="n">
+      <c r="C20" s="8" t="inlineStr"/>
+      <c r="D20" s="8" t="inlineStr"/>
+      <c r="E20" s="8" t="inlineStr"/>
+      <c r="F20" s="10" t="n">
         <v>6</v>
       </c>
-      <c r="G19" s="7" t="inlineStr"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="4" t="inlineStr">
+      <c r="G20" s="8" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
         <is>
           <t>2026-09-14</t>
         </is>
       </c>
-      <c r="B20" s="4" t="inlineStr">
+      <c r="B21" s="5" t="inlineStr">
         <is>
           <t>Disease Detection - Deployment</t>
         </is>
       </c>
-      <c r="C20" s="4" t="inlineStr">
+      <c r="C21" s="5" t="inlineStr">
         <is>
           <t>Uploaded the model, its crop list and the service that answers the app, together. Verified the live service is answering with the new model before calling it done.</t>
         </is>
       </c>
-      <c r="D20" s="4" t="inlineStr">
+      <c r="D21" s="5" t="inlineStr">
         <is>
           <t>deploy_to_space.py</t>
         </is>
       </c>
-      <c r="E20" s="5" t="inlineStr">
+      <c r="E21" s="6" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="F20" s="6" t="n">
+      <c r="F21" s="7" t="n">
         <v>1.5</v>
       </c>
-      <c r="G20" s="4" t="inlineStr">
+      <c r="G21" s="5" t="inlineStr">
         <is>
           <t>Live and confirmed: 32 classes, 9 crops, wheat and rice present. The upload script now refuses to run if the model and the crop list disagree - an earlier deployment sent the wrong model because nothing checked.</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="4" t="inlineStr">
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
         <is>
           <t>2026-09-14</t>
         </is>
       </c>
-      <c r="B21" s="4" t="inlineStr">
+      <c r="B22" s="5" t="inlineStr">
         <is>
           <t>App - Confidence Threshold</t>
         </is>
       </c>
-      <c r="C21" s="4" t="inlineStr">
+      <c r="C22" s="5" t="inlineStr">
         <is>
           <t>Raised the confidence level below which the app declines to name a disease, from 70% to 80%, measured across the same test set.</t>
         </is>
       </c>
-      <c r="D21" s="4" t="inlineStr">
+      <c r="D22" s="5" t="inlineStr">
         <is>
           <t>src/services/api.js</t>
         </is>
       </c>
-      <c r="E21" s="5" t="inlineStr">
+      <c r="E22" s="6" t="inlineStr">
         <is>
           <t>Fixed</t>
         </is>
       </c>
-      <c r="F21" s="6" t="n">
+      <c r="F22" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="G21" s="4" t="inlineStr">
+      <c r="G22" s="5" t="inlineStr">
         <is>
           <t>About a quarter fewer wrong diagnoses reach the farmer, for six points of coverage. An unanswered scan costs him another photograph; a wrong one costs him a fungicide.</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="4" t="inlineStr">
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
         <is>
           <t>2026-09-14</t>
         </is>
       </c>
-      <c r="B22" s="4" t="inlineStr">
+      <c r="B23" s="5" t="inlineStr">
         <is>
           <t>Accuracy Report</t>
         </is>
       </c>
-      <c r="C22" s="4" t="inlineStr">
+      <c r="C23" s="5" t="inlineStr">
         <is>
           <t>Prepared the accuracy report for sending, as a Word document and a web page, with the before-and-after chart by crop.</t>
         </is>
       </c>
-      <c r="D22" s="4" t="inlineStr">
+      <c r="D23" s="5" t="inlineStr">
         <is>
           <t>SmartKisan_Model_Accuracy_2026-09-14.docx / .html</t>
         </is>
       </c>
-      <c r="E22" s="5" t="inlineStr">
+      <c r="E23" s="6" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="F22" s="6" t="n">
+      <c r="F23" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="G22" s="4" t="inlineStr">
+      <c r="G23" s="5" t="inlineStr">
         <is>
           <t>Trimmed to the four headline figures, the chart, the table and the confidence threshold. How the work was done was removed; what it produced was kept.</t>
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="4" t="inlineStr">
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
         <is>
           <t>2026-09-14</t>
         </is>
       </c>
-      <c r="B23" s="4" t="inlineStr">
+      <c r="B24" s="5" t="inlineStr">
         <is>
           <t>Accuracy Report - Correction</t>
         </is>
       </c>
-      <c r="C23" s="4" t="inlineStr">
-        <is>
-          <t>Found and fixed a labelling error in our own report before sending it. The chart called our first training run the previous model, which reads as the model the app was running.</t>
-        </is>
-      </c>
-      <c r="D23" s="4" t="inlineStr">
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>Found and fixed a labelling error in my own report before sending it. The chart called my first training run the previous model, which reads as the model the app was running.</t>
+        </is>
+      </c>
+      <c r="D24" s="5" t="inlineStr">
         <is>
           <t>docs/reports/model-accuracy-2026-09-14.html</t>
         </is>
       </c>
-      <c r="E23" s="5" t="inlineStr">
+      <c r="E24" s="6" t="inlineStr">
         <is>
           <t>Fixed</t>
         </is>
       </c>
-      <c r="F23" s="6" t="n">
+      <c r="F24" s="7" t="n">
         <v>0.5</v>
       </c>
-      <c r="G23" s="4" t="inlineStr">
+      <c r="G24" s="5" t="inlineStr">
         <is>
           <t>The report was comparing against one baseline in the headline figures and a different one in the chart, under the same word. Also added the like-for-like figure, 35% to 86%, alongside the headline 28% to 87% - see the Result section below.</t>
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="4" t="inlineStr">
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
         <is>
           <t>2026-09-14</t>
         </is>
       </c>
-      <c r="B24" s="4" t="inlineStr">
+      <c r="B25" s="5" t="inlineStr">
         <is>
           <t>Test Build</t>
         </is>
       </c>
-      <c r="C24" s="4" t="inlineStr">
+      <c r="C25" s="5" t="inlineStr">
         <is>
           <t>Built a test APK. First build since 31 August, so it also carries the fixes made in between.</t>
         </is>
       </c>
-      <c r="D24" s="4" t="inlineStr">
+      <c r="D25" s="5" t="inlineStr">
         <is>
           <t>SmartKisan-test-2026-09-14.apk (71 MB)</t>
         </is>
       </c>
-      <c r="E24" s="11" t="inlineStr">
+      <c r="E25" s="12" t="inlineStr">
         <is>
           <t>Ready for Testing</t>
         </is>
       </c>
-      <c r="F24" s="6" t="n">
+      <c r="F25" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="G24" s="4" t="inlineStr">
+      <c r="G25" s="5" t="inlineStr">
         <is>
           <t>Also includes: profile edits saving, the forgot-password flow, phone one-time codes, the pump routes that were writing to database columns that do not exist, and real data behind crop suitability and farm management.</t>
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="7" t="inlineStr"/>
-      <c r="B25" s="8" t="inlineStr">
+    <row r="26">
+      <c r="A26" s="8" t="inlineStr"/>
+      <c r="B26" s="9" t="inlineStr">
         <is>
           <t>Monday 14 September - total</t>
         </is>
       </c>
-      <c r="C25" s="7" t="inlineStr"/>
-      <c r="D25" s="7" t="inlineStr"/>
-      <c r="E25" s="7" t="inlineStr"/>
-      <c r="F25" s="9" t="n">
+      <c r="C26" s="8" t="inlineStr"/>
+      <c r="D26" s="8" t="inlineStr"/>
+      <c r="E26" s="8" t="inlineStr"/>
+      <c r="F26" s="10" t="n">
         <v>6</v>
       </c>
-      <c r="G25" s="7" t="inlineStr"/>
-    </row>
-    <row r="27">
-      <c r="A27" s="12" t="inlineStr">
-        <is>
-          <t>Result - measured on 1,581 photographs never seen in training</t>
-        </is>
-      </c>
+      <c r="G26" s="8" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="13" t="inlineStr">
         <is>
+          <t>Result - measured on 1,581 photographs never seen in training</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="14" t="inlineStr">
+        <is>
           <t>Measure</t>
         </is>
       </c>
-      <c r="B28" s="13" t="inlineStr">
+      <c r="B29" s="14" t="inlineStr">
         <is>
           <t>Old model</t>
         </is>
       </c>
-      <c r="C28" s="13" t="inlineStr">
+      <c r="C29" s="14" t="inlineStr">
         <is>
           <t>Now</t>
         </is>
       </c>
-      <c r="D28" s="13" t="inlineStr">
+      <c r="D29" s="14" t="inlineStr">
         <is>
           <t>Note</t>
-        </is>
-      </c>
-      <c r="E28" t="inlineStr"/>
-      <c r="F28" t="inlineStr"/>
-      <c r="G28" t="inlineStr"/>
-    </row>
-    <row r="29">
-      <c r="A29" s="4" t="inlineStr">
-        <is>
-          <t>Disease named correctly</t>
-        </is>
-      </c>
-      <c r="B29" s="4" t="inlineStr">
-        <is>
-          <t>28%</t>
-        </is>
-      </c>
-      <c r="C29" s="5" t="inlineStr">
-        <is>
-          <t>87%</t>
-        </is>
-      </c>
-      <c r="D29" s="4" t="inlineStr">
-        <is>
-          <t>On 1,581 photographs the model never saw in training</t>
         </is>
       </c>
       <c r="E29" t="inlineStr"/>
@@ -1288,24 +1277,24 @@
       <c r="G29" t="inlineStr"/>
     </row>
     <row r="30">
-      <c r="A30" s="4" t="inlineStr">
-        <is>
-          <t>Crop named correctly</t>
-        </is>
-      </c>
-      <c r="B30" s="4" t="inlineStr">
-        <is>
-          <t>49%</t>
-        </is>
-      </c>
-      <c r="C30" s="5" t="inlineStr">
-        <is>
-          <t>99%</t>
-        </is>
-      </c>
-      <c r="D30" s="4" t="inlineStr">
-        <is>
-          <t>Which plant it is looking at</t>
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>Disease named correctly</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="inlineStr">
+        <is>
+          <t>28%</t>
+        </is>
+      </c>
+      <c r="C30" s="6" t="inlineStr">
+        <is>
+          <t>87%</t>
+        </is>
+      </c>
+      <c r="D30" s="5" t="inlineStr">
+        <is>
+          <t>On 1,581 photographs the model never saw in training</t>
         </is>
       </c>
       <c r="E30" t="inlineStr"/>
@@ -1313,24 +1302,24 @@
       <c r="G30" t="inlineStr"/>
     </row>
     <row r="31">
-      <c r="A31" s="4" t="inlineStr">
-        <is>
-          <t>Healthy plant called diseased</t>
-        </is>
-      </c>
-      <c r="B31" s="4" t="inlineStr">
-        <is>
-          <t>42%</t>
-        </is>
-      </c>
-      <c r="C31" s="5" t="inlineStr">
-        <is>
-          <t>8%</t>
-        </is>
-      </c>
-      <c r="D31" s="4" t="inlineStr">
-        <is>
-          <t>A spray recommended to a farmer who did not need one</t>
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>Crop named correctly</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="inlineStr">
+        <is>
+          <t>49%</t>
+        </is>
+      </c>
+      <c r="C31" s="6" t="inlineStr">
+        <is>
+          <t>99%</t>
+        </is>
+      </c>
+      <c r="D31" s="5" t="inlineStr">
+        <is>
+          <t>Which plant it is looking at</t>
         </is>
       </c>
       <c r="E31" t="inlineStr"/>
@@ -1338,24 +1327,24 @@
       <c r="G31" t="inlineStr"/>
     </row>
     <row r="32">
-      <c r="A32" s="4" t="inlineStr">
-        <is>
-          <t>Crops covered</t>
-        </is>
-      </c>
-      <c r="B32" s="4" t="inlineStr">
-        <is>
-          <t>7</t>
-        </is>
-      </c>
-      <c r="C32" s="5" t="inlineStr">
-        <is>
-          <t>9</t>
-        </is>
-      </c>
-      <c r="D32" s="4" t="inlineStr">
-        <is>
-          <t>Wheat and rice added - most of our users grow them</t>
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>Healthy plant called diseased</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="inlineStr">
+        <is>
+          <t>42%</t>
+        </is>
+      </c>
+      <c r="C32" s="6" t="inlineStr">
+        <is>
+          <t>8%</t>
+        </is>
+      </c>
+      <c r="D32" s="5" t="inlineStr">
+        <is>
+          <t>A spray recommended to a farmer who did not need one</t>
         </is>
       </c>
       <c r="E32" t="inlineStr"/>
@@ -1363,24 +1352,24 @@
       <c r="G32" t="inlineStr"/>
     </row>
     <row r="33">
-      <c r="A33" s="4" t="inlineStr">
-        <is>
-          <t>Tomato</t>
-        </is>
-      </c>
-      <c r="B33" s="4" t="inlineStr">
-        <is>
-          <t>44%</t>
-        </is>
-      </c>
-      <c r="C33" s="5" t="inlineStr">
-        <is>
-          <t>88%</t>
-        </is>
-      </c>
-      <c r="D33" s="4" t="inlineStr">
-        <is>
-          <t>Before figure is our own first training run</t>
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>Crops covered</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="C33" s="6" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="D33" s="5" t="inlineStr">
+        <is>
+          <t>Wheat and rice added - most SmartKisan users grow them</t>
         </is>
       </c>
       <c r="E33" t="inlineStr"/>
@@ -1388,24 +1377,24 @@
       <c r="G33" t="inlineStr"/>
     </row>
     <row r="34">
-      <c r="A34" s="4" t="inlineStr">
-        <is>
-          <t>Potato</t>
-        </is>
-      </c>
-      <c r="B34" s="4" t="inlineStr">
-        <is>
-          <t>50%</t>
-        </is>
-      </c>
-      <c r="C34" s="5" t="inlineStr">
-        <is>
-          <t>86%</t>
-        </is>
-      </c>
-      <c r="D34" s="4" t="inlineStr">
-        <is>
-          <t>Before figure is our own first training run</t>
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>Tomato</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="inlineStr">
+        <is>
+          <t>44%</t>
+        </is>
+      </c>
+      <c r="C34" s="6" t="inlineStr">
+        <is>
+          <t>88%</t>
+        </is>
+      </c>
+      <c r="D34" s="5" t="inlineStr">
+        <is>
+          <t>Before figure is my first training run</t>
         </is>
       </c>
       <c r="E34" t="inlineStr"/>
@@ -1413,24 +1402,24 @@
       <c r="G34" t="inlineStr"/>
     </row>
     <row r="35">
-      <c r="A35" s="4" t="inlineStr">
-        <is>
-          <t>Maize</t>
-        </is>
-      </c>
-      <c r="B35" s="4" t="inlineStr">
-        <is>
-          <t>65%</t>
-        </is>
-      </c>
-      <c r="C35" s="5" t="inlineStr">
-        <is>
-          <t>82%</t>
-        </is>
-      </c>
-      <c r="D35" s="4" t="inlineStr">
-        <is>
-          <t>Before figure is our own first training run</t>
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>Potato</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="inlineStr">
+        <is>
+          <t>50%</t>
+        </is>
+      </c>
+      <c r="C35" s="6" t="inlineStr">
+        <is>
+          <t>86%</t>
+        </is>
+      </c>
+      <c r="D35" s="5" t="inlineStr">
+        <is>
+          <t>Before figure is my first training run</t>
         </is>
       </c>
       <c r="E35" t="inlineStr"/>
@@ -1438,24 +1427,24 @@
       <c r="G35" t="inlineStr"/>
     </row>
     <row r="36">
-      <c r="A36" s="4" t="inlineStr">
-        <is>
-          <t>Rice</t>
-        </is>
-      </c>
-      <c r="B36" s="4" t="inlineStr">
-        <is>
-          <t>not covered</t>
-        </is>
-      </c>
-      <c r="C36" s="5" t="inlineStr">
-        <is>
-          <t>92%</t>
-        </is>
-      </c>
-      <c r="D36" s="4" t="inlineStr">
-        <is>
-          <t>The old model had no rice class</t>
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>Maize</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="inlineStr">
+        <is>
+          <t>65%</t>
+        </is>
+      </c>
+      <c r="C36" s="6" t="inlineStr">
+        <is>
+          <t>82%</t>
+        </is>
+      </c>
+      <c r="D36" s="5" t="inlineStr">
+        <is>
+          <t>Before figure is my first training run</t>
         </is>
       </c>
       <c r="E36" t="inlineStr"/>
@@ -1463,24 +1452,24 @@
       <c r="G36" t="inlineStr"/>
     </row>
     <row r="37">
-      <c r="A37" s="4" t="inlineStr">
-        <is>
-          <t>Wheat</t>
-        </is>
-      </c>
-      <c r="B37" s="4" t="inlineStr">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>Rice</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="inlineStr">
         <is>
           <t>not covered</t>
         </is>
       </c>
-      <c r="C37" s="5" t="inlineStr">
-        <is>
-          <t>90%</t>
-        </is>
-      </c>
-      <c r="D37" s="4" t="inlineStr">
-        <is>
-          <t>The old model had no wheat class</t>
+      <c r="C37" s="6" t="inlineStr">
+        <is>
+          <t>92%</t>
+        </is>
+      </c>
+      <c r="D37" s="5" t="inlineStr">
+        <is>
+          <t>The old model had no rice class</t>
         </is>
       </c>
       <c r="E37" t="inlineStr"/>
@@ -1488,63 +1477,71 @@
       <c r="G37" t="inlineStr"/>
     </row>
     <row r="38">
-      <c r="A38" s="4" t="inlineStr">
-        <is>
-          <t>Like-for-like</t>
-        </is>
-      </c>
-      <c r="B38" s="4" t="inlineStr">
-        <is>
-          <t>about 35%</t>
-        </is>
-      </c>
-      <c r="C38" s="5" t="inlineStr">
-        <is>
-          <t>about 86%</t>
-        </is>
-      </c>
-      <c r="D38" s="4" t="inlineStr">
-        <is>
-          <t>A fifth of the test set is rice and wheat, which the old model could never have answered. Excluding those, this is the fair comparison. Both numbers are real; the farmer experiences 28% to 87%.</t>
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="inlineStr">
+        <is>
+          <t>not covered</t>
+        </is>
+      </c>
+      <c r="C38" s="6" t="inlineStr">
+        <is>
+          <t>90%</t>
+        </is>
+      </c>
+      <c r="D38" s="5" t="inlineStr">
+        <is>
+          <t>The old model had no wheat class</t>
         </is>
       </c>
       <c r="E38" t="inlineStr"/>
       <c r="F38" t="inlineStr"/>
       <c r="G38" t="inlineStr"/>
     </row>
-    <row r="40">
-      <c r="A40" s="12" t="inlineStr">
-        <is>
-          <t>Why this took three days and not one</t>
-        </is>
-      </c>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t>Like-for-like</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="inlineStr">
+        <is>
+          <t>about 35%</t>
+        </is>
+      </c>
+      <c r="C39" s="6" t="inlineStr">
+        <is>
+          <t>about 86%</t>
+        </is>
+      </c>
+      <c r="D39" s="5" t="inlineStr">
+        <is>
+          <t>A fifth of the test set is rice and wheat, which the old model could never have answered. Excluding those, this is the fair comparison. Both numbers are real; the farmer experiences 28% to 87%.</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr"/>
+      <c r="F39" t="inlineStr"/>
+      <c r="G39" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" s="13" t="inlineStr">
         <is>
+          <t>Why this took three days and not one</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="14" t="inlineStr">
+        <is>
           <t>Reason</t>
         </is>
       </c>
-      <c r="B41" s="13" t="inlineStr">
+      <c r="B42" s="14" t="inlineStr">
         <is>
           <t>Detail</t>
-        </is>
-      </c>
-      <c r="C41" t="inlineStr"/>
-      <c r="D41" t="inlineStr"/>
-      <c r="E41" t="inlineStr"/>
-      <c r="F41" t="inlineStr"/>
-      <c r="G41" t="inlineStr"/>
-    </row>
-    <row r="42">
-      <c r="A42" s="4" t="inlineStr">
-        <is>
-          <t>Training time</t>
-        </is>
-      </c>
-      <c r="B42" s="4" t="inlineStr">
-        <is>
-          <t>One full training run takes about five hours on a laptop processor. We have no graphics card. Three runs were needed, so roughly 15 of the 18 hours was the machine working.</t>
         </is>
       </c>
       <c r="C42" t="inlineStr"/>
@@ -1554,14 +1551,14 @@
       <c r="G42" t="inlineStr"/>
     </row>
     <row r="43">
-      <c r="A43" s="4" t="inlineStr">
-        <is>
-          <t>Runs cannot overlap</t>
-        </is>
-      </c>
-      <c r="B43" s="4" t="inlineStr">
-        <is>
-          <t>Running two at once was tried. Both slowed badly - one step went from 8 minutes to 37. So it is one run at a time.</t>
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t>Training time</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="inlineStr">
+        <is>
+          <t>One full training run takes about five hours on a laptop processor. I have no graphics card, and I needed three runs, so roughly 15 of the 18 hours was the machine working rather than me.</t>
         </is>
       </c>
       <c r="C43" t="inlineStr"/>
@@ -1571,14 +1568,14 @@
       <c r="G43" t="inlineStr"/>
     </row>
     <row r="44">
-      <c r="A44" s="4" t="inlineStr">
-        <is>
-          <t>Results arrive only at the end</t>
-        </is>
-      </c>
-      <c r="B44" s="4" t="inlineStr">
-        <is>
-          <t>Whether a change worked is unknown until the run finishes. The shape of the day is: start a run, wait, measure, work out what went wrong, change one thing, start the next. Two attempts a day at most.</t>
+      <c r="A44" s="5" t="inlineStr">
+        <is>
+          <t>Runs cannot overlap</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="inlineStr">
+        <is>
+          <t>I tried running two at once. Both slowed badly - one step went from 8 minutes to 37. So it is one run at a time.</t>
         </is>
       </c>
       <c r="C44" t="inlineStr"/>
@@ -1588,14 +1585,14 @@
       <c r="G44" t="inlineStr"/>
     </row>
     <row r="45">
-      <c r="A45" s="4" t="inlineStr">
-        <is>
-          <t>Two of the three runs failed</t>
-        </is>
-      </c>
-      <c r="B45" s="4" t="inlineStr">
-        <is>
-          <t>That is the part that was worth the time. The failed rebalancing run is what proved the problem was field conditions and not a shortage of data. Without it, the next day would have been spent adding more of the wrong thing.</t>
+      <c r="A45" s="5" t="inlineStr">
+        <is>
+          <t>Results arrive only at the end</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="inlineStr">
+        <is>
+          <t>Whether a change worked is unknown until the run finishes. My day is: start a run, wait, measure, work out what went wrong, change one thing, start the next. Two attempts a day at most.</t>
         </is>
       </c>
       <c r="C45" t="inlineStr"/>
@@ -1605,14 +1602,14 @@
       <c r="G45" t="inlineStr"/>
     </row>
     <row r="46">
-      <c r="A46" s="4" t="inlineStr">
-        <is>
-          <t>What would make it faster</t>
-        </is>
-      </c>
-      <c r="B46" s="4" t="inlineStr">
-        <is>
-          <t>Renting a cloud graphics card for a day brings a five-hour run to well under an hour. The same job would fit in one shift instead of three.</t>
+      <c r="A46" s="5" t="inlineStr">
+        <is>
+          <t>Two of the three runs failed</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="inlineStr">
+        <is>
+          <t>That is the part that was worth the time. The failed rebalancing run is what proved the problem was field conditions and not a shortage of data. Without it, I would have spent the next day adding more of the wrong thing.</t>
         </is>
       </c>
       <c r="C46" t="inlineStr"/>
@@ -1621,48 +1618,44 @@
       <c r="F46" t="inlineStr"/>
       <c r="G46" t="inlineStr"/>
     </row>
-    <row r="48">
-      <c r="A48" s="12" t="inlineStr">
-        <is>
-          <t>Open Items</t>
-        </is>
-      </c>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t>What would make it faster</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="inlineStr">
+        <is>
+          <t>Renting a cloud graphics card for a day brings a five-hour run to well under an hour. The same job would fit into one of my shifts instead of three.</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr"/>
+      <c r="D47" t="inlineStr"/>
+      <c r="E47" t="inlineStr"/>
+      <c r="F47" t="inlineStr"/>
+      <c r="G47" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" s="13" t="inlineStr">
         <is>
+          <t>Open Items</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="14" t="inlineStr">
+        <is>
           <t>Reference</t>
         </is>
       </c>
-      <c r="B49" s="13" t="inlineStr">
+      <c r="B50" s="14" t="inlineStr">
         <is>
           <t>Item</t>
         </is>
       </c>
-      <c r="C49" s="13" t="inlineStr">
+      <c r="C50" s="14" t="inlineStr">
         <is>
           <t>Blocked On / Next Step</t>
-        </is>
-      </c>
-      <c r="D49" t="inlineStr"/>
-      <c r="E49" t="inlineStr"/>
-      <c r="F49" t="inlineStr"/>
-      <c r="G49" t="inlineStr"/>
-    </row>
-    <row r="50">
-      <c r="A50" s="4" t="inlineStr">
-        <is>
-          <t>Disease model</t>
-        </is>
-      </c>
-      <c r="B50" s="4" t="inlineStr">
-        <is>
-          <t>Field testing not yet done</t>
-        </is>
-      </c>
-      <c r="C50" s="4" t="inlineStr">
-        <is>
-          <t>Tomato, potato and maize are measured mostly on collections where we divided training and testing images ourselves, so those are the optimistic end. On the one collection where outside authors published the division, the model scores 57%. Real field results will land between the two.</t>
         </is>
       </c>
       <c r="D50" t="inlineStr"/>
@@ -1671,19 +1664,19 @@
       <c r="G50" t="inlineStr"/>
     </row>
     <row r="51">
-      <c r="A51" s="4" t="inlineStr">
-        <is>
-          <t>Weed model</t>
-        </is>
-      </c>
-      <c r="B51" s="4" t="inlineStr">
-        <is>
-          <t>Grass weeds identified 13% of the time</t>
-        </is>
-      </c>
-      <c r="C51" s="4" t="inlineStr">
-        <is>
-          <t>Unchanged from the 3 September report and still the priority for weed work. Grass against broadleaf decides which herbicide is bought, so this matters more than the overall figure.</t>
+      <c r="A51" s="5" t="inlineStr">
+        <is>
+          <t>Disease model</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="inlineStr">
+        <is>
+          <t>Field testing not yet done</t>
+        </is>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>Tomato, potato and maize are measured mostly on collections where I divided the training and testing images myself, so those are the optimistic end. On the one collection where outside authors published the division, the model scores 57%. Real field results will land between the two.</t>
         </is>
       </c>
       <c r="D51" t="inlineStr"/>
@@ -1692,19 +1685,19 @@
       <c r="G51" t="inlineStr"/>
     </row>
     <row r="52">
-      <c r="A52" s="4" t="inlineStr">
-        <is>
-          <t>Training hardware</t>
-        </is>
-      </c>
-      <c r="B52" s="4" t="inlineStr">
-        <is>
-          <t>No graphics card</t>
-        </is>
-      </c>
-      <c r="C52" s="4" t="inlineStr">
-        <is>
-          <t>The main reason this work is measured in days rather than hours. A rented cloud machine for a day would remove it.</t>
+      <c r="A52" s="5" t="inlineStr">
+        <is>
+          <t>Weed model</t>
+        </is>
+      </c>
+      <c r="B52" s="5" t="inlineStr">
+        <is>
+          <t>Grass weeds identified 13% of the time</t>
+        </is>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>Unchanged from the 3 September report and still the priority for weed work. Grass against broadleaf decides which herbicide is bought, so this matters more than the overall figure.</t>
         </is>
       </c>
       <c r="D52" t="inlineStr"/>
@@ -1713,19 +1706,19 @@
       <c r="G52" t="inlineStr"/>
     </row>
     <row r="53">
-      <c r="A53" s="4" t="inlineStr">
-        <is>
-          <t>Phone sign-in</t>
-        </is>
-      </c>
-      <c r="B53" s="4" t="inlineStr">
-        <is>
-          <t>Codes cannot reach Indian numbers</t>
-        </is>
-      </c>
-      <c r="C53" s="4" t="inlineStr">
-        <is>
-          <t>Unchanged. Requires DLT registration with TRAI, or credentials for an SMS account the company already holds. Business registration, not development.</t>
+      <c r="A53" s="5" t="inlineStr">
+        <is>
+          <t>Training hardware</t>
+        </is>
+      </c>
+      <c r="B53" s="5" t="inlineStr">
+        <is>
+          <t>No graphics card</t>
+        </is>
+      </c>
+      <c r="C53" s="5" t="inlineStr">
+        <is>
+          <t>The main reason this work is measured in days rather than hours. A rented cloud machine for a day would remove it, and I would not need three shifts for the next model.</t>
         </is>
       </c>
       <c r="D53" t="inlineStr"/>
@@ -1734,19 +1727,19 @@
       <c r="G53" t="inlineStr"/>
     </row>
     <row r="54">
-      <c r="A54" s="4" t="inlineStr">
-        <is>
-          <t>Real-time messaging</t>
-        </is>
-      </c>
-      <c r="B54" s="4" t="inlineStr">
-        <is>
-          <t>Pump control uses a public broker</t>
-        </is>
-      </c>
-      <c r="C54" s="4" t="inlineStr">
-        <is>
-          <t>Unchanged. Anyone who knows a user ID could read sensor data or switch a pump. Needs a private broker before physical hardware is connected.</t>
+      <c r="A54" s="5" t="inlineStr">
+        <is>
+          <t>Phone sign-in</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="inlineStr">
+        <is>
+          <t>Codes cannot reach Indian numbers</t>
+        </is>
+      </c>
+      <c r="C54" s="5" t="inlineStr">
+        <is>
+          <t>Unchanged. Requires DLT registration with TRAI, or credentials for an SMS account the company already holds. Business registration, not development.</t>
         </is>
       </c>
       <c r="D54" t="inlineStr"/>
@@ -1754,13 +1747,35 @@
       <c r="F54" t="inlineStr"/>
       <c r="G54" t="inlineStr"/>
     </row>
+    <row r="55">
+      <c r="A55" s="5" t="inlineStr">
+        <is>
+          <t>Real-time messaging</t>
+        </is>
+      </c>
+      <c r="B55" s="5" t="inlineStr">
+        <is>
+          <t>Pump control uses a public broker</t>
+        </is>
+      </c>
+      <c r="C55" s="5" t="inlineStr">
+        <is>
+          <t>Unchanged. Anyone who knows a user ID could read sensor data or switch a pump. Needs a private broker before physical hardware is connected.</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr"/>
+      <c r="E55" t="inlineStr"/>
+      <c r="F55" t="inlineStr"/>
+      <c r="G55" t="inlineStr"/>
+    </row>
   </sheetData>
-  <mergeCells count="5">
+  <mergeCells count="6">
     <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A40:G40"/>
-    <mergeCell ref="A27:G27"/>
-    <mergeCell ref="A48:G48"/>
+    <mergeCell ref="A3:G3"/>
     <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A41:G41"/>
+    <mergeCell ref="A49:G49"/>
+    <mergeCell ref="A28:G28"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>